<commit_message>
Updated data dictionary: Added Dictionary and Table Explanation
</commit_message>
<xml_diff>
--- a/Design/data_dictionary.xlsx
+++ b/Design/data_dictionary.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://binusianorg-my.sharepoint.com/personal/muhammad_prasetya007_binus_ac_id/Documents/Kuliah/Project Portofolio/ecommerce-database/Design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="91" documentId="8_{A57C5DB2-1096-44F3-8168-754811DA2E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22DFDAFB-E955-544E-ABC8-C37C14B8BD52}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="8_{A57C5DB2-1096-44F3-8168-754811DA2E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC1E48D6-23BF-44CC-9611-60CC3BEFD730}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA73638C-C858-472B-AEA7-A7EFEA41F37E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Dictionary" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
   <si>
     <t>Products</t>
   </si>
@@ -137,7 +135,31 @@
     <t>Order Item</t>
   </si>
   <si>
-    <t>Table Explanation</t>
+    <t>Tabel yang menyimpan setiap item yang diorder</t>
+  </si>
+  <si>
+    <t>Tabel yang menyimpan setiap order yang dilakukan</t>
+  </si>
+  <si>
+    <t>Tabel yang menyimpan data metode pembayaran yang tersedia</t>
+  </si>
+  <si>
+    <t>Tabel yang menyimpan identitas kasir yang melayani transaksi</t>
+  </si>
+  <si>
+    <t>Tabel yang menyimpan voucher untuk diskon transaksi</t>
+  </si>
+  <si>
+    <t>Tabel yang menyimpan toko yang tersedia</t>
+  </si>
+  <si>
+    <t>Tabel yang menyimpan produk yang tersedia</t>
+  </si>
+  <si>
+    <t>Payment Category</t>
+  </si>
+  <si>
+    <t>Entity Explanation</t>
   </si>
 </sst>
 </file>
@@ -153,7 +175,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -162,18 +184,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -181,14 +197,61 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -206,10 +269,14 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -247,7 +314,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -353,7 +420,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -495,7 +562,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -503,211 +570,226 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD9BCB96-3D1F-43F8-9AB2-983D98EE6559}">
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.66015625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.37109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.59765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.71875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="3.44140625" customWidth="1"/>
+    <col min="9" max="9" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="53.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>28</v>
       </c>
+      <c r="I1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J1" s="4"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="I2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>29</v>
       </c>
+      <c r="I3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F5" s="1"/>
+      <c r="G5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>30</v>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="I7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="I8" s="1" t="s">
         <v>28</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I1:J1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated data_dictionary.xlsx: Reordered dictionary
</commit_message>
<xml_diff>
--- a/Design/data_dictionary.xlsx
+++ b/Design/data_dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://binusianorg-my.sharepoint.com/personal/muhammad_prasetya007_binus_ac_id/Documents/Kuliah/Project Portofolio/ecommerce-database/Design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="132" documentId="8_{A57C5DB2-1096-44F3-8168-754811DA2E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC1E48D6-23BF-44CC-9611-60CC3BEFD730}"/>
+  <xr:revisionPtr revIDLastSave="141" documentId="8_{A57C5DB2-1096-44F3-8168-754811DA2E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47208D29-4857-414D-9C2E-608A37DF8851}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA73638C-C858-472B-AEA7-A7EFEA41F37E}"/>
   </bookViews>
@@ -573,13 +573,13 @@
   <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="3.44140625" customWidth="1"/>
     <col min="9" max="9" width="15.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="53.33203125" bestFit="1" customWidth="1"/>
@@ -593,19 +593,19 @@
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>41</v>
@@ -620,19 +620,19 @@
         <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>1</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>5</v>
@@ -646,22 +646,22 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>0</v>
@@ -675,22 +675,22 @@
         <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>32</v>
@@ -704,20 +704,20 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>14</v>
@@ -729,18 +729,18 @@
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>24</v>
@@ -752,14 +752,14 @@
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="C7" s="1"/>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="I7" s="1" t="s">
         <v>2</v>
@@ -772,11 +772,11 @@
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="I8" s="1" t="s">
         <v>28</v>

</xml_diff>